<commit_message>
Introduce JSON-based database seeding system
Replaces legacy Excel seeding with typed C# seeders reading from JSON files in Seeder/SeedData. Adds seed models, orchestrators, and DI registration. Includes dev tools for Excel-to-JSON export and SQLite seed testing. Updates README and project config. Marks ExcelSeeder as obsolete; legacy Excel file retained for migration reference. Seeders operate in "if empty" mode for safety.
</commit_message>
<xml_diff>
--- a/backend/API/SeedData.xlsx
+++ b/backend/API/SeedData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jakub\Desktop\Cs\pc\RestaurantOrderingAppSolution\backend\API\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Piccolo\RestaurantOrderingAppSolution\backend\API\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7E014274-5C7C-4C20-8514-8C45313A6EAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCD072AE-DC05-44C4-8831-126886657FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="4" xr2:uid="{C8CF7BA1-E9AA-4852-A9EB-5F1AD6BFABCB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="12" xr2:uid="{C8CF7BA1-E9AA-4852-A9EB-5F1AD6BFABCB}"/>
   </bookViews>
   <sheets>
     <sheet name="CustomerInformation" sheetId="1" r:id="rId1"/>
@@ -19,12 +19,12 @@
     <sheet name="SubCategory" sheetId="4" r:id="rId4"/>
     <sheet name="MenuItem" sheetId="5" r:id="rId5"/>
     <sheet name="Table" sheetId="7" r:id="rId6"/>
-    <sheet name="Tag" sheetId="8" r:id="rId7"/>
-    <sheet name="Reservation" sheetId="9" r:id="rId8"/>
-    <sheet name="OrderItem" sheetId="10" r:id="rId9"/>
-    <sheet name="Order" sheetId="11" r:id="rId10"/>
-    <sheet name="MenuItemIngredientRel" sheetId="6" r:id="rId11"/>
-    <sheet name="Area" sheetId="13" r:id="rId12"/>
+    <sheet name="Reservation" sheetId="9" r:id="rId7"/>
+    <sheet name="OrderItem" sheetId="10" r:id="rId8"/>
+    <sheet name="Order" sheetId="11" r:id="rId9"/>
+    <sheet name="MenuItemIngredientRel" sheetId="6" r:id="rId10"/>
+    <sheet name="Area" sheetId="13" r:id="rId11"/>
+    <sheet name="Tag" sheetId="8" r:id="rId12"/>
     <sheet name="IngredientTagRel" sheetId="12" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1576" uniqueCount="398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1576" uniqueCount="385">
   <si>
     <t>Id</t>
   </si>
@@ -856,45 +856,6 @@
   </si>
   <si>
     <t>TagId</t>
-  </si>
-  <si>
-    <t>e3e07ec9-75f1-45bb-b435-7ab002a68b74</t>
-  </si>
-  <si>
-    <t>e3e07ec9-75f1-45bb-b435-7ab002a68b75</t>
-  </si>
-  <si>
-    <t>e3e07ec9-75f1-45bb-b435-7ab002a68b76</t>
-  </si>
-  <si>
-    <t>e3e07ec9-75f1-45bb-b435-7ab002a68b77</t>
-  </si>
-  <si>
-    <t>15febb8e-5c89-4416-ac10-7011f7f31cd9</t>
-  </si>
-  <si>
-    <t>15febb8e-5c89-4416-ac10-7011f7f31cd10</t>
-  </si>
-  <si>
-    <t>15febb8e-5c89-4416-ac10-7011f7f31cd11</t>
-  </si>
-  <si>
-    <t>15febb8e-5c89-4416-ac10-7011f7f31cd12</t>
-  </si>
-  <si>
-    <t>66109b01-6f01-49e9-ab47-249eba53f078</t>
-  </si>
-  <si>
-    <t>66109b01-6f01-49e9-ab47-249eba53f079</t>
-  </si>
-  <si>
-    <t>66109b01-6f01-49e9-ab47-249eba53f080</t>
-  </si>
-  <si>
-    <t>66109b01-6f01-49e9-ab47-249eba53f081</t>
-  </si>
-  <si>
-    <t>66109b01-6f01-49e9-ab47-249eba53f082</t>
   </si>
   <si>
     <t>5ecdc81b-929e-4ee9-b82d-8a7d4f3218a6</t>
@@ -1316,7 +1277,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1372,12 +1333,6 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1397,9 +1352,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Motyw pakietu Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Motyw pakietu Office 2013–2022">
   <a:themeElements>
-    <a:clrScheme name="Pakiet Office">
+    <a:clrScheme name="Pakiet Office 2013–2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1437,7 +1392,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Pakiet Office">
+    <a:fontScheme name="Pakiet Office 2013–2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1543,7 +1498,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Pakiet Office">
+    <a:fmtScheme name="Pakiet Office 2013–2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1685,7 +1640,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1795,141 +1750,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA4966BB-B585-4EFD-A171-2B6D26A10B97}">
-  <dimension ref="A1:I4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="36.5703125" customWidth="1"/>
-    <col min="2" max="2" width="23.140625" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" customWidth="1"/>
-    <col min="8" max="8" width="37.42578125" customWidth="1"/>
-    <col min="9" max="9" width="36.42578125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
-      <c r="A2" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="10">
-        <v>45726.604166666664</v>
-      </c>
-      <c r="C2" s="2">
-        <v>30</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2">
-        <v>0</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
-      <c r="A3" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" s="10">
-        <v>45757.618055555555</v>
-      </c>
-      <c r="C3" s="2">
-        <v>40</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2">
-        <v>0</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="B4" s="10">
-        <v>45758.618055555555</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0</v>
-      </c>
-      <c r="E4" s="2">
-        <v>0</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D2E4AC9-0CD2-4F25-AD3B-36A84397D079}">
   <dimension ref="A1:T224"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2144,7 +1964,7 @@
         <v>147</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>396</v>
+        <v>383</v>
       </c>
       <c r="M19" s="8"/>
       <c r="N19" s="12"/>
@@ -2391,7 +2211,7 @@
         <v>150</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>396</v>
+        <v>383</v>
       </c>
       <c r="M38" s="8"/>
       <c r="N38" s="12"/>
@@ -4270,7 +4090,7 @@
     </row>
     <row r="190" spans="1:2">
       <c r="A190" s="2" t="s">
-        <v>387</v>
+        <v>374</v>
       </c>
       <c r="B190" s="1" t="s">
         <v>12</v>
@@ -4278,7 +4098,7 @@
     </row>
     <row r="191" spans="1:2">
       <c r="A191" s="2" t="s">
-        <v>387</v>
+        <v>374</v>
       </c>
       <c r="B191" s="2" t="s">
         <v>66</v>
@@ -4286,7 +4106,7 @@
     </row>
     <row r="192" spans="1:2">
       <c r="A192" s="2" t="s">
-        <v>387</v>
+        <v>374</v>
       </c>
       <c r="B192" s="2" t="s">
         <v>76</v>
@@ -4294,7 +4114,7 @@
     </row>
     <row r="193" spans="1:2">
       <c r="A193" s="2" t="s">
-        <v>387</v>
+        <v>374</v>
       </c>
       <c r="B193" s="2" t="s">
         <v>85</v>
@@ -4302,7 +4122,7 @@
     </row>
     <row r="194" spans="1:2">
       <c r="A194" s="2" t="s">
-        <v>387</v>
+        <v>374</v>
       </c>
       <c r="B194" s="2" t="s">
         <v>72</v>
@@ -4310,7 +4130,7 @@
     </row>
     <row r="195" spans="1:2">
       <c r="A195" s="2" t="s">
-        <v>387</v>
+        <v>374</v>
       </c>
       <c r="B195" s="2" t="s">
         <v>70</v>
@@ -4318,7 +4138,7 @@
     </row>
     <row r="196" spans="1:2">
       <c r="A196" s="2" t="s">
-        <v>388</v>
+        <v>375</v>
       </c>
       <c r="B196" s="1" t="s">
         <v>12</v>
@@ -4326,7 +4146,7 @@
     </row>
     <row r="197" spans="1:2">
       <c r="A197" s="2" t="s">
-        <v>388</v>
+        <v>375</v>
       </c>
       <c r="B197" s="2" t="s">
         <v>66</v>
@@ -4334,7 +4154,7 @@
     </row>
     <row r="198" spans="1:2">
       <c r="A198" s="2" t="s">
-        <v>388</v>
+        <v>375</v>
       </c>
       <c r="B198" s="2" t="s">
         <v>76</v>
@@ -4342,7 +4162,7 @@
     </row>
     <row r="199" spans="1:2">
       <c r="A199" s="2" t="s">
-        <v>388</v>
+        <v>375</v>
       </c>
       <c r="B199" s="2" t="s">
         <v>77</v>
@@ -4350,7 +4170,7 @@
     </row>
     <row r="200" spans="1:2">
       <c r="A200" s="2" t="s">
-        <v>388</v>
+        <v>375</v>
       </c>
       <c r="B200" s="2" t="s">
         <v>83</v>
@@ -4358,7 +4178,7 @@
     </row>
     <row r="201" spans="1:2">
       <c r="A201" s="2" t="s">
-        <v>388</v>
+        <v>375</v>
       </c>
       <c r="B201" s="2" t="s">
         <v>90</v>
@@ -4366,7 +4186,7 @@
     </row>
     <row r="202" spans="1:2">
       <c r="A202" s="2" t="s">
-        <v>389</v>
+        <v>376</v>
       </c>
       <c r="B202" s="2" t="s">
         <v>66</v>
@@ -4374,7 +4194,7 @@
     </row>
     <row r="203" spans="1:2">
       <c r="A203" s="2" t="s">
-        <v>389</v>
+        <v>376</v>
       </c>
       <c r="B203" s="1" t="s">
         <v>11</v>
@@ -4382,7 +4202,7 @@
     </row>
     <row r="204" spans="1:2">
       <c r="A204" s="2" t="s">
-        <v>389</v>
+        <v>376</v>
       </c>
       <c r="B204" s="2" t="s">
         <v>79</v>
@@ -4390,7 +4210,7 @@
     </row>
     <row r="205" spans="1:2">
       <c r="A205" s="2" t="s">
-        <v>389</v>
+        <v>376</v>
       </c>
       <c r="B205" s="2" t="s">
         <v>88</v>
@@ -4398,7 +4218,7 @@
     </row>
     <row r="206" spans="1:2">
       <c r="A206" s="2" t="s">
-        <v>389</v>
+        <v>376</v>
       </c>
       <c r="B206" s="2" t="s">
         <v>68</v>
@@ -4406,7 +4226,7 @@
     </row>
     <row r="207" spans="1:2">
       <c r="A207" s="2" t="s">
-        <v>390</v>
+        <v>377</v>
       </c>
       <c r="B207" s="1" t="s">
         <v>12</v>
@@ -4414,7 +4234,7 @@
     </row>
     <row r="208" spans="1:2">
       <c r="A208" s="2" t="s">
-        <v>390</v>
+        <v>377</v>
       </c>
       <c r="B208" s="2" t="s">
         <v>66</v>
@@ -4422,7 +4242,7 @@
     </row>
     <row r="209" spans="1:2">
       <c r="A209" s="2" t="s">
-        <v>390</v>
+        <v>377</v>
       </c>
       <c r="B209" s="2" t="s">
         <v>80</v>
@@ -4430,7 +4250,7 @@
     </row>
     <row r="210" spans="1:2">
       <c r="A210" s="2" t="s">
-        <v>390</v>
+        <v>377</v>
       </c>
       <c r="B210" s="2" t="s">
         <v>67</v>
@@ -4438,7 +4258,7 @@
     </row>
     <row r="211" spans="1:2">
       <c r="A211" s="2" t="s">
-        <v>390</v>
+        <v>377</v>
       </c>
       <c r="B211" s="2" t="s">
         <v>84</v>
@@ -4446,7 +4266,7 @@
     </row>
     <row r="212" spans="1:2">
       <c r="A212" s="2" t="s">
-        <v>390</v>
+        <v>377</v>
       </c>
       <c r="B212" s="2" t="s">
         <v>95</v>
@@ -4454,7 +4274,7 @@
     </row>
     <row r="213" spans="1:2">
       <c r="A213" s="2" t="s">
-        <v>391</v>
+        <v>378</v>
       </c>
       <c r="B213" s="1" t="s">
         <v>12</v>
@@ -4462,7 +4282,7 @@
     </row>
     <row r="214" spans="1:2">
       <c r="A214" s="2" t="s">
-        <v>391</v>
+        <v>378</v>
       </c>
       <c r="B214" s="2" t="s">
         <v>66</v>
@@ -4470,7 +4290,7 @@
     </row>
     <row r="215" spans="1:2">
       <c r="A215" s="2" t="s">
-        <v>391</v>
+        <v>378</v>
       </c>
       <c r="B215" s="2" t="s">
         <v>75</v>
@@ -4478,7 +4298,7 @@
     </row>
     <row r="216" spans="1:2">
       <c r="A216" s="2" t="s">
-        <v>391</v>
+        <v>378</v>
       </c>
       <c r="B216" s="2" t="s">
         <v>87</v>
@@ -4486,7 +4306,7 @@
     </row>
     <row r="217" spans="1:2">
       <c r="A217" s="2" t="s">
-        <v>391</v>
+        <v>378</v>
       </c>
       <c r="B217" s="2" t="s">
         <v>99</v>
@@ -4494,7 +4314,7 @@
     </row>
     <row r="218" spans="1:2">
       <c r="A218" s="2" t="s">
-        <v>391</v>
+        <v>378</v>
       </c>
       <c r="B218" s="2" t="s">
         <v>73</v>
@@ -4502,7 +4322,7 @@
     </row>
     <row r="219" spans="1:2">
       <c r="A219" s="2" t="s">
-        <v>392</v>
+        <v>379</v>
       </c>
       <c r="B219" s="1" t="s">
         <v>12</v>
@@ -4510,7 +4330,7 @@
     </row>
     <row r="220" spans="1:2">
       <c r="A220" s="2" t="s">
-        <v>392</v>
+        <v>379</v>
       </c>
       <c r="B220" s="2" t="s">
         <v>66</v>
@@ -4518,7 +4338,7 @@
     </row>
     <row r="221" spans="1:2">
       <c r="A221" s="2" t="s">
-        <v>392</v>
+        <v>379</v>
       </c>
       <c r="B221" s="2" t="s">
         <v>81</v>
@@ -4526,7 +4346,7 @@
     </row>
     <row r="222" spans="1:2">
       <c r="A222" s="2" t="s">
-        <v>392</v>
+        <v>379</v>
       </c>
       <c r="B222" s="2" t="s">
         <v>83</v>
@@ -4534,7 +4354,7 @@
     </row>
     <row r="223" spans="1:2">
       <c r="A223" s="2" t="s">
-        <v>392</v>
+        <v>379</v>
       </c>
       <c r="B223" s="2" t="s">
         <v>86</v>
@@ -4542,7 +4362,7 @@
     </row>
     <row r="224" spans="1:2">
       <c r="A224" s="2" t="s">
-        <v>392</v>
+        <v>379</v>
       </c>
       <c r="B224" s="2" t="s">
         <v>96</v>
@@ -4554,7 +4374,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17577034-6810-45EB-B138-D5219A90AFAB}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -4580,10 +4400,10 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
-        <v>283</v>
+        <v>270</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>288</v>
+        <v>275</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>64</v>
@@ -4594,10 +4414,10 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
-        <v>284</v>
+        <v>271</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>289</v>
+        <v>276</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>64</v>
@@ -4608,10 +4428,10 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>290</v>
+        <v>277</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>64</v>
@@ -4622,10 +4442,10 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2" t="s">
-        <v>286</v>
+        <v>273</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>291</v>
+        <v>278</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>64</v>
@@ -4636,15 +4456,140 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2" t="s">
-        <v>287</v>
+        <v>274</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>64</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DEDC361-D738-4510-89A2-AB67CB12EBDF}">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="41.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>65</v>
       </c>
     </row>
@@ -4739,7 +4684,7 @@
         <v>72</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>274</v>
+        <v>241</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -4747,7 +4692,7 @@
         <v>73</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>275</v>
+        <v>241</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -4811,7 +4756,7 @@
         <v>81</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>278</v>
+        <v>246</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -4819,7 +4764,7 @@
         <v>82</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>279</v>
+        <v>246</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -4827,7 +4772,7 @@
         <v>83</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>280</v>
+        <v>246</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -4835,7 +4780,7 @@
         <v>84</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>281</v>
+        <v>246</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -4843,7 +4788,7 @@
         <v>85</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>282</v>
+        <v>246</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -4899,7 +4844,7 @@
         <v>92</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>274</v>
+        <v>241</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -4907,7 +4852,7 @@
         <v>93</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>275</v>
+        <v>241</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -4915,7 +4860,7 @@
         <v>94</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>276</v>
+        <v>241</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -4923,7 +4868,7 @@
         <v>95</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>277</v>
+        <v>241</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -4939,7 +4884,7 @@
         <v>97</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>270</v>
+        <v>245</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -4947,7 +4892,7 @@
         <v>98</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>271</v>
+        <v>245</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -4955,7 +4900,7 @@
         <v>99</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>272</v>
+        <v>245</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -4963,12 +4908,12 @@
         <v>100</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>273</v>
+        <v>245</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2" t="s">
-        <v>396</v>
+        <v>383</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>244</v>
@@ -5652,10 +5597,10 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="2" t="s">
-        <v>396</v>
+        <v>383</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>395</v>
+        <v>382</v>
       </c>
       <c r="C39" s="2">
         <v>5</v>
@@ -5699,7 +5644,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>397</v>
+        <v>384</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -5889,8 +5834,8 @@
       <c r="E1" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="F1" s="20" t="s">
-        <v>397</v>
+      <c r="F1" s="2" t="s">
+        <v>384</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -5909,7 +5854,7 @@
       <c r="E2" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="F2" s="21">
+      <c r="F2" s="19">
         <v>1</v>
       </c>
     </row>
@@ -5929,7 +5874,7 @@
       <c r="E3" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="F3" s="21">
+      <c r="F3" s="19">
         <v>2</v>
       </c>
     </row>
@@ -5949,7 +5894,7 @@
       <c r="E4" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="F4" s="21">
+      <c r="F4" s="19">
         <v>3</v>
       </c>
     </row>
@@ -5969,7 +5914,7 @@
       <c r="E5" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="F5" s="21">
+      <c r="F5" s="19">
         <v>4</v>
       </c>
     </row>
@@ -5989,7 +5934,7 @@
       <c r="E6" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="F6" s="21">
+      <c r="F6" s="19">
         <v>5</v>
       </c>
     </row>
@@ -6009,7 +5954,7 @@
       <c r="E7" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="F7" s="21">
+      <c r="F7" s="19">
         <v>6</v>
       </c>
     </row>
@@ -6029,7 +5974,7 @@
       <c r="E8" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="F8" s="21">
+      <c r="F8" s="19">
         <v>7</v>
       </c>
     </row>
@@ -6049,7 +5994,7 @@
       <c r="E9" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="F9" s="21">
+      <c r="F9" s="19">
         <v>8</v>
       </c>
     </row>
@@ -6098,8 +6043,8 @@
       <c r="H1" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="I1" s="19" t="s">
-        <v>397</v>
+      <c r="I1" s="1" t="s">
+        <v>384</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -6107,7 +6052,7 @@
         <v>144</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>300</v>
+        <v>287</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>185</v>
@@ -6136,7 +6081,7 @@
         <v>145</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>315</v>
+        <v>302</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>185</v>
@@ -6165,7 +6110,7 @@
         <v>146</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>301</v>
+        <v>288</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>185</v>
@@ -6194,7 +6139,7 @@
         <v>147</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>324</v>
+        <v>311</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>185</v>
@@ -6223,7 +6168,7 @@
         <v>148</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>325</v>
+        <v>312</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>185</v>
@@ -6252,7 +6197,7 @@
         <v>149</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>302</v>
+        <v>289</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>185</v>
@@ -6281,7 +6226,7 @@
         <v>150</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>316</v>
+        <v>303</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>185</v>
@@ -6310,7 +6255,7 @@
         <v>151</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>303</v>
+        <v>290</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>185</v>
@@ -6339,7 +6284,7 @@
         <v>152</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>326</v>
+        <v>313</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>185</v>
@@ -6368,7 +6313,7 @@
         <v>153</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>327</v>
+        <v>314</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>185</v>
@@ -6397,7 +6342,7 @@
         <v>154</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>328</v>
+        <v>315</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>185</v>
@@ -6426,7 +6371,7 @@
         <v>155</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>304</v>
+        <v>291</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>185</v>
@@ -6455,7 +6400,7 @@
         <v>156</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>305</v>
+        <v>292</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>185</v>
@@ -6484,7 +6429,7 @@
         <v>157</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>306</v>
+        <v>293</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>185</v>
@@ -6513,7 +6458,7 @@
         <v>158</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>307</v>
+        <v>294</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>185</v>
@@ -6542,7 +6487,7 @@
         <v>159</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>308</v>
+        <v>295</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>185</v>
@@ -6571,7 +6516,7 @@
         <v>160</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>317</v>
+        <v>304</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>185</v>
@@ -6600,7 +6545,7 @@
         <v>161</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>318</v>
+        <v>305</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>185</v>
@@ -6629,7 +6574,7 @@
         <v>162</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>319</v>
+        <v>306</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>185</v>
@@ -6658,7 +6603,7 @@
         <v>163</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>309</v>
+        <v>296</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>185</v>
@@ -6687,7 +6632,7 @@
         <v>164</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>310</v>
+        <v>297</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>185</v>
@@ -6716,7 +6661,7 @@
         <v>165</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>320</v>
+        <v>307</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>185</v>
@@ -6745,7 +6690,7 @@
         <v>166</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>311</v>
+        <v>298</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>185</v>
@@ -6774,7 +6719,7 @@
         <v>167</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>321</v>
+        <v>308</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>185</v>
@@ -6803,7 +6748,7 @@
         <v>168</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>312</v>
+        <v>299</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>185</v>
@@ -6832,7 +6777,7 @@
         <v>169</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>335</v>
+        <v>322</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>143</v>
@@ -6861,7 +6806,7 @@
         <v>170</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>322</v>
+        <v>309</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>185</v>
@@ -6890,7 +6835,7 @@
         <v>171</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>313</v>
+        <v>300</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>185</v>
@@ -6919,7 +6864,7 @@
         <v>172</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>329</v>
+        <v>316</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>185</v>
@@ -6948,7 +6893,7 @@
         <v>173</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>314</v>
+        <v>301</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>185</v>
@@ -6977,7 +6922,7 @@
         <v>174</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>323</v>
+        <v>310</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>185</v>
@@ -7151,7 +7096,7 @@
         <v>180</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>330</v>
+        <v>317</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>185</v>
@@ -7180,7 +7125,7 @@
         <v>181</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>331</v>
+        <v>318</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>185</v>
@@ -7209,7 +7154,7 @@
         <v>182</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>332</v>
+        <v>319</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>185</v>
@@ -7238,7 +7183,7 @@
         <v>183</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>333</v>
+        <v>320</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>185</v>
@@ -7267,7 +7212,7 @@
         <v>184</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>334</v>
+        <v>321</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>143</v>
@@ -7325,7 +7270,7 @@
         <v>188</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>367</v>
+        <v>354</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>143</v>
@@ -7354,7 +7299,7 @@
         <v>189</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>348</v>
+        <v>335</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>143</v>
@@ -7383,7 +7328,7 @@
         <v>190</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>350</v>
+        <v>337</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>143</v>
@@ -7470,7 +7415,7 @@
         <v>195</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>336</v>
+        <v>323</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>143</v>
@@ -7499,7 +7444,7 @@
         <v>196</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>337</v>
+        <v>324</v>
       </c>
       <c r="C50" s="13" t="s">
         <v>143</v>
@@ -7525,10 +7470,10 @@
     </row>
     <row r="51" spans="1:9">
       <c r="A51" s="2" t="s">
-        <v>368</v>
+        <v>355</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>338</v>
+        <v>325</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>143</v>
@@ -7554,10 +7499,10 @@
     </row>
     <row r="52" spans="1:9">
       <c r="A52" s="2" t="s">
-        <v>369</v>
+        <v>356</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>339</v>
+        <v>326</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>143</v>
@@ -7583,10 +7528,10 @@
     </row>
     <row r="53" spans="1:9">
       <c r="A53" s="2" t="s">
-        <v>370</v>
+        <v>357</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>340</v>
+        <v>327</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>143</v>
@@ -7612,10 +7557,10 @@
     </row>
     <row r="54" spans="1:9">
       <c r="A54" s="2" t="s">
-        <v>371</v>
+        <v>358</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>341</v>
+        <v>328</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>143</v>
@@ -7641,10 +7586,10 @@
     </row>
     <row r="55" spans="1:9">
       <c r="A55" s="2" t="s">
-        <v>372</v>
+        <v>359</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>342</v>
+        <v>329</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>143</v>
@@ -7670,10 +7615,10 @@
     </row>
     <row r="56" spans="1:9">
       <c r="A56" s="2" t="s">
-        <v>373</v>
+        <v>360</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>343</v>
+        <v>330</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>143</v>
@@ -7699,10 +7644,10 @@
     </row>
     <row r="57" spans="1:9">
       <c r="A57" s="2" t="s">
-        <v>374</v>
+        <v>361</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>344</v>
+        <v>331</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>143</v>
@@ -7728,10 +7673,10 @@
     </row>
     <row r="58" spans="1:9">
       <c r="A58" s="2" t="s">
-        <v>375</v>
+        <v>362</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>345</v>
+        <v>332</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>143</v>
@@ -7757,10 +7702,10 @@
     </row>
     <row r="59" spans="1:9">
       <c r="A59" s="2" t="s">
-        <v>376</v>
+        <v>363</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>346</v>
+        <v>333</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>143</v>
@@ -7786,10 +7731,10 @@
     </row>
     <row r="60" spans="1:9">
       <c r="A60" s="2" t="s">
-        <v>377</v>
+        <v>364</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>347</v>
+        <v>334</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>143</v>
@@ -7815,10 +7760,10 @@
     </row>
     <row r="61" spans="1:9">
       <c r="A61" s="2" t="s">
-        <v>378</v>
+        <v>365</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>143</v>
@@ -7844,10 +7789,10 @@
     </row>
     <row r="62" spans="1:9">
       <c r="A62" s="2" t="s">
-        <v>379</v>
+        <v>366</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>349</v>
+        <v>336</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>143</v>
@@ -7873,10 +7818,10 @@
     </row>
     <row r="63" spans="1:9">
       <c r="A63" s="2" t="s">
-        <v>380</v>
+        <v>367</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>363</v>
+        <v>350</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>143</v>
@@ -7902,10 +7847,10 @@
     </row>
     <row r="64" spans="1:9">
       <c r="A64" s="2" t="s">
-        <v>381</v>
+        <v>368</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>351</v>
+        <v>338</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>143</v>
@@ -7931,10 +7876,10 @@
     </row>
     <row r="65" spans="1:9">
       <c r="A65" s="2" t="s">
-        <v>382</v>
+        <v>369</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>352</v>
+        <v>339</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>143</v>
@@ -7960,10 +7905,10 @@
     </row>
     <row r="66" spans="1:9">
       <c r="A66" s="2" t="s">
-        <v>383</v>
+        <v>370</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>353</v>
+        <v>340</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>143</v>
@@ -7989,10 +7934,10 @@
     </row>
     <row r="67" spans="1:9">
       <c r="A67" s="2" t="s">
-        <v>384</v>
+        <v>371</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>354</v>
+        <v>341</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>143</v>
@@ -8018,10 +7963,10 @@
     </row>
     <row r="68" spans="1:9">
       <c r="A68" s="2" t="s">
-        <v>385</v>
+        <v>372</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>355</v>
+        <v>342</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>143</v>
@@ -8047,10 +7992,10 @@
     </row>
     <row r="69" spans="1:9">
       <c r="A69" s="2" t="s">
-        <v>386</v>
+        <v>373</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>356</v>
+        <v>343</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>143</v>
@@ -8076,10 +8021,10 @@
     </row>
     <row r="70" spans="1:9">
       <c r="A70" s="2" t="s">
-        <v>387</v>
+        <v>374</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>357</v>
+        <v>344</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>185</v>
@@ -8105,10 +8050,10 @@
     </row>
     <row r="71" spans="1:9">
       <c r="A71" s="2" t="s">
-        <v>388</v>
+        <v>375</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>358</v>
+        <v>345</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>185</v>
@@ -8134,10 +8079,10 @@
     </row>
     <row r="72" spans="1:9">
       <c r="A72" s="2" t="s">
-        <v>389</v>
+        <v>376</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>359</v>
+        <v>346</v>
       </c>
       <c r="C72" s="1" t="s">
         <v>185</v>
@@ -8163,10 +8108,10 @@
     </row>
     <row r="73" spans="1:9">
       <c r="A73" s="2" t="s">
-        <v>390</v>
+        <v>377</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>360</v>
+        <v>347</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>185</v>
@@ -8192,10 +8137,10 @@
     </row>
     <row r="74" spans="1:9">
       <c r="A74" s="2" t="s">
-        <v>391</v>
+        <v>378</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>361</v>
+        <v>348</v>
       </c>
       <c r="C74" s="1" t="s">
         <v>185</v>
@@ -8221,10 +8166,10 @@
     </row>
     <row r="75" spans="1:9">
       <c r="A75" s="2" t="s">
-        <v>392</v>
+        <v>379</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>362</v>
+        <v>349</v>
       </c>
       <c r="C75" s="1" t="s">
         <v>185</v>
@@ -8250,10 +8195,10 @@
     </row>
     <row r="76" spans="1:9">
       <c r="A76" s="2" t="s">
-        <v>393</v>
+        <v>380</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>364</v>
+        <v>351</v>
       </c>
       <c r="C76" s="2" t="s">
         <v>143</v>
@@ -8279,10 +8224,10 @@
     </row>
     <row r="77" spans="1:9">
       <c r="A77" s="2" t="s">
-        <v>394</v>
+        <v>381</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>365</v>
+        <v>352</v>
       </c>
       <c r="C77" s="2" t="s">
         <v>143</v>
@@ -8345,7 +8290,7 @@
         <v>200</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>292</v>
+        <v>279</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -8368,7 +8313,7 @@
         <v>264</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>283</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -8391,7 +8336,7 @@
         <v>223</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>283</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -8414,7 +8359,7 @@
         <v>223</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>283</v>
+        <v>270</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -8437,7 +8382,7 @@
         <v>223</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>283</v>
+        <v>270</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -8460,7 +8405,7 @@
         <v>223</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>284</v>
+        <v>271</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -8483,7 +8428,7 @@
         <v>223</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>284</v>
+        <v>271</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -8506,7 +8451,7 @@
         <v>223</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>284</v>
+        <v>271</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -8529,7 +8474,7 @@
         <v>223</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>284</v>
+        <v>271</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -8552,7 +8497,7 @@
         <v>223</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>286</v>
+        <v>273</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -8575,7 +8520,7 @@
         <v>223</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>286</v>
+        <v>273</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -8598,7 +8543,7 @@
         <v>223</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>286</v>
+        <v>273</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -8621,7 +8566,7 @@
         <v>223</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>286</v>
+        <v>273</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -8644,7 +8589,7 @@
         <v>223</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>287</v>
+        <v>274</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -8667,7 +8612,7 @@
         <v>223</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>287</v>
+        <v>274</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -8690,7 +8635,7 @@
         <v>223</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>287</v>
+        <v>274</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -8713,7 +8658,7 @@
         <v>223</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>287</v>
+        <v>274</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -8736,7 +8681,7 @@
         <v>223</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>287</v>
+        <v>274</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -8759,15 +8704,15 @@
         <v>223</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>287</v>
+        <v>274</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="2" t="s">
-        <v>296</v>
+        <v>283</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>293</v>
+        <v>280</v>
       </c>
       <c r="C20" s="2">
         <v>4</v>
@@ -8782,15 +8727,15 @@
         <v>223</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="2" t="s">
-        <v>297</v>
+        <v>284</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>294</v>
+        <v>281</v>
       </c>
       <c r="C21" s="2">
         <v>4</v>
@@ -8805,15 +8750,15 @@
         <v>223</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="2" t="s">
-        <v>298</v>
+        <v>285</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>295</v>
+        <v>282</v>
       </c>
       <c r="C22" s="2">
         <v>2</v>
@@ -8828,7 +8773,7 @@
         <v>223</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
     </row>
   </sheetData>
@@ -8837,131 +8782,6 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DEDC361-D738-4510-89A2-AB67CB12EBDF}">
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="36.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F05608C-89F7-443B-8F02-A238CB7CF577}">
   <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -9048,7 +8868,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C9E1B61-911D-4E67-9431-CC6DC22C7D98}">
   <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -9131,4 +8951,139 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA4966BB-B585-4EFD-A171-2B6D26A10B97}">
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="36.5703125" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" customWidth="1"/>
+    <col min="8" max="8" width="37.42578125" customWidth="1"/>
+    <col min="9" max="9" width="36.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="10">
+        <v>45726.604166666664</v>
+      </c>
+      <c r="C2" s="2">
+        <v>30</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0</v>
+      </c>
+      <c r="E2" s="2">
+        <v>0</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="10">
+        <v>45757.618055555555</v>
+      </c>
+      <c r="C3" s="2">
+        <v>40</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="B4" s="10">
+        <v>45758.618055555555</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0</v>
+      </c>
+      <c r="E4" s="2">
+        <v>0</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>